<commit_message>
add battery runtime calcs
</commit_message>
<xml_diff>
--- a/TECH_DOCS/Battery_Sizing_Calculation.xlsx
+++ b/TECH_DOCS/Battery_Sizing_Calculation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dawn3\Documents\Projects\MATERIAL_TRANSFER_ROBOT_2026\TECH_DOCS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ECE4A5D-3994-43E2-85D4-865936FBCAF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CDF73F6-B8DA-4B63-9EF5-5B7FA73C9183}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EAE27284-3B62-4067-A50A-96499FEC82D4}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
   <si>
     <t>Drive Motors</t>
   </si>
@@ -81,9 +81,6 @@
   </si>
   <si>
     <t>Speaker</t>
-  </si>
-  <si>
-    <t>WiFi Module</t>
   </si>
   <si>
     <t>LIDAR</t>
@@ -238,11 +235,11 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -577,7 +574,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCEEB80E-F96E-4A81-8664-353830E8CFBC}">
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.5546875" bestFit="1" customWidth="1"/>
@@ -592,18 +589,18 @@
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="7"/>
       <c r="B1" s="7"/>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8" t="s">
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="10"/>
+      <c r="J1" s="10"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -613,10 +610,10 @@
         <v>3</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>18</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>19</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>4</v>
@@ -628,7 +625,7 @@
         <v>8</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>5</v>
@@ -637,7 +634,7 @@
         <v>6</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
@@ -653,8 +650,8 @@
         <v>12</v>
       </c>
       <c r="F3" s="2">
-        <f>SUM(F4:F8)</f>
-        <v>32.4</v>
+        <f>SUM(F4:F7)</f>
+        <v>32.15</v>
       </c>
       <c r="G3" s="2">
         <v>11.1</v>
@@ -664,15 +661,15 @@
       </c>
       <c r="I3" s="2">
         <f>F3/H3</f>
-        <v>38.117647058823529</v>
+        <v>37.823529411764703</v>
       </c>
       <c r="J3" s="2">
         <f>I3/G3</f>
-        <v>3.4340222575516695</v>
+        <v>3.4075251722310544</v>
       </c>
       <c r="K3" s="2">
         <f>J3*15%</f>
-        <v>0.51510333863275037</v>
+        <v>0.5111287758346581</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
@@ -714,7 +711,7 @@
         <v>5</v>
       </c>
       <c r="F5" s="3">
-        <f t="shared" ref="F5:F8" si="0">E5*C5*B5</f>
+        <f t="shared" ref="F5:F7" si="0">E5*C5*B5</f>
         <v>10</v>
       </c>
       <c r="G5" s="4"/>
@@ -755,7 +752,7 @@
         <v>1</v>
       </c>
       <c r="C7" s="3">
-        <v>0.05</v>
+        <v>0.38</v>
       </c>
       <c r="D7" s="4"/>
       <c r="E7" s="3">
@@ -763,7 +760,7 @@
       </c>
       <c r="F7" s="3">
         <f t="shared" si="0"/>
-        <v>0.25</v>
+        <v>1.9</v>
       </c>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -772,115 +769,115 @@
       <c r="K7" s="4"/>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A8" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" s="3">
-        <v>1</v>
-      </c>
-      <c r="C8" s="3">
-        <v>0.38</v>
-      </c>
-      <c r="D8" s="4"/>
-      <c r="E8" s="3">
-        <v>5</v>
-      </c>
-      <c r="F8" s="3">
-        <f t="shared" si="0"/>
-        <v>1.9</v>
-      </c>
-      <c r="G8" s="4"/>
+      <c r="A8" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B8" s="2">
+        <v>2</v>
+      </c>
+      <c r="C8" s="2">
+        <v>1.37</v>
+      </c>
+      <c r="D8" s="2">
+        <v>15</v>
+      </c>
+      <c r="E8" s="2">
+        <v>12</v>
+      </c>
+      <c r="F8" s="2">
+        <f t="shared" ref="F8" si="1">B8*C8*E8</f>
+        <v>32.880000000000003</v>
+      </c>
+      <c r="G8" s="2">
+        <v>11.1</v>
+      </c>
       <c r="H8" s="4"/>
-      <c r="I8" s="4"/>
-      <c r="J8" s="4"/>
+      <c r="I8" s="2">
+        <f>F8</f>
+        <v>32.880000000000003</v>
+      </c>
+      <c r="J8" s="2">
+        <f>I8/G8</f>
+        <v>2.9621621621621625</v>
+      </c>
       <c r="K8" s="4"/>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="B9" s="2">
         <v>2</v>
       </c>
-      <c r="C9" s="2">
-        <v>1.37</v>
-      </c>
-      <c r="D9" s="2">
-        <v>15</v>
-      </c>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
       <c r="E9" s="2">
         <v>12</v>
       </c>
       <c r="F9" s="2">
-        <f t="shared" ref="F9" si="1">B9*C9*E9</f>
-        <v>32.880000000000003</v>
+        <f>SUM(F10:F12)</f>
+        <v>0.92500000000000004</v>
       </c>
       <c r="G9" s="2">
         <v>11.1</v>
       </c>
-      <c r="H9" s="4"/>
+      <c r="H9" s="2">
+        <v>0.97</v>
+      </c>
       <c r="I9" s="2">
-        <f>F9</f>
-        <v>32.880000000000003</v>
+        <f>F9/H9</f>
+        <v>0.95360824742268047</v>
       </c>
       <c r="J9" s="2">
         <f>I9/G9</f>
-        <v>2.9621621621621625</v>
-      </c>
-      <c r="K9" s="4"/>
+        <v>8.5910652920962213E-2</v>
+      </c>
+      <c r="K9" s="2">
+        <f>J9*3%</f>
+        <v>2.5773195876288664E-3</v>
+      </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10" s="2">
-        <v>1</v>
-      </c>
-      <c r="C10" s="4"/>
+      <c r="A10" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="3">
+        <v>2</v>
+      </c>
+      <c r="C10" s="3">
+        <v>1.4999999999999999E-2</v>
+      </c>
       <c r="D10" s="4"/>
-      <c r="E10" s="2">
-        <v>12</v>
-      </c>
-      <c r="F10" s="2">
-        <f>SUM(F11:F13)</f>
-        <v>1.0250000000000001</v>
-      </c>
-      <c r="G10" s="2">
-        <v>11.1</v>
-      </c>
-      <c r="H10" s="2">
-        <v>0.97</v>
-      </c>
-      <c r="I10" s="2">
-        <f>F10/H10</f>
-        <v>1.0567010309278353</v>
-      </c>
-      <c r="J10" s="2">
-        <f>I10/G10</f>
-        <v>9.5198291074579763E-2</v>
-      </c>
-      <c r="K10" s="2">
-        <f>J10*3%</f>
-        <v>2.8559487322373928E-3</v>
-      </c>
+      <c r="E10" s="3">
+        <v>5</v>
+      </c>
+      <c r="F10" s="3">
+        <f>E10*C10*B10</f>
+        <v>0.15</v>
+      </c>
+      <c r="G10" s="4"/>
+      <c r="H10" s="4"/>
+      <c r="I10" s="4"/>
+      <c r="J10" s="4"/>
+      <c r="K10" s="4"/>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>20</v>
       </c>
       <c r="B11" s="3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C11" s="3">
-        <v>1.4999999999999999E-2</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="D11" s="4"/>
       <c r="E11" s="3">
         <v>5</v>
       </c>
       <c r="F11" s="3">
-        <f>E11*C11*B11</f>
-        <v>0.3</v>
+        <f t="shared" ref="F11:F12" si="2">E11*C11*B11</f>
+        <v>7.5000000000000011E-2</v>
       </c>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -893,18 +890,18 @@
         <v>21</v>
       </c>
       <c r="B12" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C12" s="3">
-        <v>5.0000000000000001E-3</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="D12" s="4"/>
       <c r="E12" s="3">
         <v>5</v>
       </c>
       <c r="F12" s="3">
-        <f t="shared" ref="F12:F13" si="2">E12*C12*B12</f>
-        <v>2.5000000000000001E-2</v>
+        <f t="shared" si="2"/>
+        <v>0.70000000000000007</v>
       </c>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -913,82 +910,58 @@
       <c r="K12" s="4"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A13" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B13" s="3">
-        <v>2</v>
-      </c>
-      <c r="C13" s="3">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="D13" s="4"/>
-      <c r="E13" s="3">
-        <v>5</v>
-      </c>
-      <c r="F13" s="3">
-        <f t="shared" si="2"/>
-        <v>0.70000000000000007</v>
-      </c>
-      <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
-      <c r="I13" s="4"/>
-      <c r="J13" s="4"/>
-      <c r="K13" s="4"/>
+      <c r="I13" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="J13" s="5">
+        <f>SUM(J3:J9)</f>
+        <v>6.4555979873141789</v>
+      </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="I14" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="J14" s="5">
-        <f>SUM(J3:J10)</f>
-        <v>6.491382710788411</v>
+      <c r="I14" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="J14" s="6">
+        <f>J13+(J13*30%)</f>
+        <v>8.3922773835084321</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="I15" s="6" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="J15" s="6">
-        <f>J14+(J14*30%)</f>
-        <v>8.4387975240249347</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="K15" s="8"/>
+      <c r="L15" s="8"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="I16" s="6" t="s">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="J16" s="6">
-        <v>10</v>
-      </c>
-      <c r="K16" s="9"/>
-      <c r="L16" s="9"/>
+        <f>J14/J15</f>
+        <v>0.83922773835084319</v>
+      </c>
     </row>
     <row r="17" spans="9:10" x14ac:dyDescent="0.3">
       <c r="I17" s="6" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="J17" s="6">
-        <f>J15/J16</f>
-        <v>0.84387975240249347</v>
+        <f>((E8*D8*B8)/G8)/J15</f>
+        <v>3.2432432432432434</v>
       </c>
     </row>
     <row r="18" spans="9:10" x14ac:dyDescent="0.3">
       <c r="I18" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="J18" s="6">
-        <f>((E9*D9*B9)/G9)/J16</f>
-        <v>3.2432432432432434</v>
-      </c>
-    </row>
-    <row r="19" spans="9:10" x14ac:dyDescent="0.3">
-      <c r="I19" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="J19" s="10">
-        <f>(J16*80%)/J15</f>
-        <v>0.94800236375198066</v>
+        <v>27</v>
+      </c>
+      <c r="J18" s="9">
+        <f>(J15*80%)/J14</f>
+        <v>0.95325733819531611</v>
       </c>
     </row>
   </sheetData>

</xml_diff>